<commit_message>
Sanity import file, lorem product copy, centred bars, demo cart by default
- content/lamgold-import.tar.gz: the sheet's content + photos for
  `npx sanity dataset import` (rebuild with npm run content:export)
- Product descriptions are two-sentence lorem ipsum placeholders
- Header bar, Add To Cart / enquiry / checkout bars: text vertically centred
- Without a Shopify token, Add To Cart always adds demo lines (checkout
  disabled), including the dev placeholder products

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0127xeMpGkamVbLsP2vpcTNu
</commit_message>
<xml_diff>
--- a/content/lamgold-content.xlsx
+++ b/content/lamgold-content.xlsx
@@ -1643,7 +1643,7 @@
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>A classic curb chain with flattened, interlocking links that lie flat against the skin with precision-cut facets on the links that increase light reflection and sparkle. Comprised of 9K gold, this timeless necklace has a width of 1 millimetres, length of 42 centimetres and weighs 1.4 grams.</t>
+          <t>Lorem ipsum dolor sit amet, consectetur adipiscing elit, sed do eiusmod tempor incididunt ut labore et dolore magna aliqua. Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</t>
         </is>
       </c>
       <c r="J2" s="7" t="inlineStr">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>A classic curb chain with flattened, interlocking links and precision-cut facets that catch the light. Comprised of 9K gold, this timeless necklace has a width of 2.1 millimetres, length of 50 centimetres and weighs 1.4 grams.</t>
+          <t>Duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur. Excepteur sint occaecat cupidatat non proident, sunt in culpa qui officia deserunt mollit anim id est laborum.</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>A classic Figaro chain with the signature pattern of short links followed by one elongated link, cut finely for a delicate line. Comprised of 9K gold, this timeless necklace has a width of 1 millimetres, length of 42 centimetres and weighs 1.4 grams.</t>
+          <t>Sed ut perspiciatis unde omnis iste natus error sit voluptatem accusantium doloremque laudantium, totam rem aperiam. Nemo enim ipsam voluptatem quia voluptas sit aspernatur aut odit aut fugit, sed quia consequuntur magni dolores.</t>
         </is>
       </c>
       <c r="J4" s="7" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>A classic Figaro chain with the signature pattern of short links followed by one elongated link, with diamond-cut facets. Comprised of 9K gold, this timeless necklace has a width of 2.1 millimetres, length of 50 centimetres and weighs 1.4 grams.</t>
+          <t>Lorem ipsum dolor sit amet, consectetur adipiscing elit, sed do eiusmod tempor incididunt ut labore et dolore magna aliqua. Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>A classic Figaro chain with the signature pattern of short links followed by one elongated link, with diamond-cut facets for extra brilliance. Comprised of 9K gold, this timeless necklace has a width of 3.3 millimetres, length of 50 centimetres and weighs 1.4 grams.</t>
+          <t>Duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur. Excepteur sint occaecat cupidatat non proident, sunt in culpa qui officia deserunt mollit anim id est laborum.</t>
         </is>
       </c>
       <c r="J6" s="7" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>A classic Chopin link chain with fine, tightly woven links that sit softly against the skin. Comprised of 14K gold, this timeless necklace has a width of 0.85 millimetres, length of 42 centimetres and weighs 1.4 grams.</t>
+          <t>Sed ut perspiciatis unde omnis iste natus error sit voluptatem accusantium doloremque laudantium, totam rem aperiam. Nemo enim ipsam voluptatem quia voluptas sit aspernatur aut odit aut fugit, sed quia consequuntur magni dolores.</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>A classic Singapore chain with twisted, diamond-cut links that ripple and catch the light with every movement. Comprised of 9K gold, this timeless necklace has a width of 1.8 millimetres, length of 42 centimetres and weighs 1.4 grams.</t>
+          <t>Lorem ipsum dolor sit amet, consectetur adipiscing elit, sed do eiusmod tempor incididunt ut labore et dolore magna aliqua. Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>A classic herringbone chain with flat, slanted links that lie smooth against the skin like a ribbon of gold. Comprised of 14K gold, this timeless necklace has a width of 1.6 millimetres, length of 42 centimetres and weighs 1.4 grams.</t>
+          <t>Duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur. Excepteur sint occaecat cupidatat non proident, sunt in culpa qui officia deserunt mollit anim id est laborum.</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>A classic box chain with square links joined edge to edge for a clean, structured line. Comprised of 9K gold, this timeless necklace has a width of 1.2 millimetres, length of 42 centimetres and weighs 1.4 grams.</t>
+          <t>Sed ut perspiciatis unde omnis iste natus error sit voluptatem accusantium doloremque laudantium, totam rem aperiam. Nemo enim ipsam voluptatem quia voluptas sit aspernatur aut odit aut fugit, sed quia consequuntur magni dolores.</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>A classic cable chain with flattened oval links that reflect light along their polished faces. Comprised of 14K gold, this timeless necklace has a width of 1 millimetres, length of 42 centimetres and weighs 1.4 grams.</t>
+          <t>Lorem ipsum dolor sit amet, consectetur adipiscing elit, sed do eiusmod tempor incididunt ut labore et dolore magna aliqua. Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>A classic anchor chain with curbed oval links each divided by a centre bar. Comprised of 9K gold, this timeless necklace has a width of 2.4 millimetres, length of 42 centimetres and weighs 1.4 grams.</t>
+          <t>Duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur. Excepteur sint occaecat cupidatat non proident, sunt in culpa qui officia deserunt mollit anim id est laborum.</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>A Gothic letter pendant in 9K gold with crisp edges and a polished face. Each initial weighs 0.8 grams and threads onto any of our chains.</t>
+          <t>Sed ut perspiciatis unde omnis iste natus error sit voluptatem accusantium doloremque laudantium, totam rem aperiam. Nemo enim ipsam voluptatem quia voluptas sit aspernatur aut odit aut fugit, sed quia consequuntur magni dolores.</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>A Figaro chain bracelet featuring the signature pattern of several short links followed by one elongated link, with diamond-cut facets added for extra brilliance and texture. Comprised of 9K gold, this timeless bracelet has a width of 2.1 millimetres, length of 16 centimetres and weighs 1.4 grams.</t>
+          <t>Lorem ipsum dolor sit amet, consectetur adipiscing elit, sed do eiusmod tempor incididunt ut labore et dolore magna aliqua. Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</t>
         </is>
       </c>
       <c r="J14" s="7" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>A Figaro chain bracelet featuring the signature pattern of several short links followed by one elongated link, with diamond-cut facets added for extra brilliance and texture. Comprised of 9K gold, this timeless bracelet has a width of 2.8 millimetres, length of 16 centimetres and weighs 1.4 grams.</t>
+          <t>Duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur. Excepteur sint occaecat cupidatat non proident, sunt in culpa qui officia deserunt mollit anim id est laborum.</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>A Figaro chain bracelet featuring the signature pattern of several short links followed by one elongated link, with diamond-cut facets added for extra brilliance and texture. Comprised of 9K gold, this timeless bracelet has a width of 3.3 millimetres, length of 16 centimetres and weighs 1.4 grams.</t>
+          <t>Sed ut perspiciatis unde omnis iste natus error sit voluptatem accusantium doloremque laudantium, totam rem aperiam. Nemo enim ipsam voluptatem quia voluptas sit aspernatur aut odit aut fugit, sed quia consequuntur magni dolores.</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>A herringbone bracelet with flat, slanted links that sit smooth against the wrist. Comprised of 14K gold, this timeless bracelet has a width of 1.5 millimetres, length of 16 centimetres and weighs 1.4 grams.</t>
+          <t>Lorem ipsum dolor sit amet, consectetur adipiscing elit, sed do eiusmod tempor incididunt ut labore et dolore magna aliqua. Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>A bevelled curb bracelet with diamond-cut, interlocking links that catch the light. Comprised of 9K gold, this timeless bracelet has a width of 2.8 millimetres, length of 16 centimetres and weighs 1.4 grams.</t>
+          <t>Duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur. Excepteur sint occaecat cupidatat non proident, sunt in culpa qui officia deserunt mollit anim id est laborum.</t>
         </is>
       </c>
       <c r="J18" s="7" t="inlineStr">
@@ -2570,7 +2570,7 @@
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>A bevelled curb bracelet with diamond-cut, interlocking links that catch the light. Comprised of 9K gold, this timeless bracelet has a width of 4.1 millimetres, length of 16 centimetres and weighs 1.4 grams.</t>
+          <t>Sed ut perspiciatis unde omnis iste natus error sit voluptatem accusantium doloremque laudantium, totam rem aperiam. Nemo enim ipsam voluptatem quia voluptas sit aspernatur aut odit aut fugit, sed quia consequuntur magni dolores.</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>A solid gold hoop earring, with streamlined clasp and symmetrical form rendered in ultra-polished gold for unparalleled brilliance. Comprised of 14K gold, this earring has a width of 3 millimetres, diameter of 16 millimetres and weighs 1.4 grams.</t>
+          <t>Lorem ipsum dolor sit amet, consectetur adipiscing elit, sed do eiusmod tempor incididunt ut labore et dolore magna aliqua. Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</t>
         </is>
       </c>
       <c r="J20" s="7" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>A solid gold hoop earring, with streamlined clasp and symmetrical form rendered in ultra-polished gold for unparalleled brilliance. Comprised of 14K gold, this earring has a width of 3 millimetres, diameter of 22 millimetres and weighs 1.4 grams.</t>
+          <t>Duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur. Excepteur sint occaecat cupidatat non proident, sunt in culpa qui officia deserunt mollit anim id est laborum.</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>A fine gold hoop earring with a seamless, lightweight form. Comprised of 14K gold, this earring has a width of 1.2 millimetres, diameter of 30 millimetres and weighs 1.4 grams.</t>
+          <t>Sed ut perspiciatis unde omnis iste natus error sit voluptatem accusantium doloremque laudantium, totam rem aperiam. Nemo enim ipsam voluptatem quia voluptas sit aspernatur aut odit aut fugit, sed quia consequuntur magni dolores.</t>
         </is>
       </c>
       <c r="J22" s="7" t="inlineStr">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>A fine gold hoop earring with a seamless, lightweight form. Comprised of 14K gold, this earring has a width of 1.2 millimetres, diameter of 50 millimetres and weighs 1.4 grams.</t>
+          <t>Lorem ipsum dolor sit amet, consectetur adipiscing elit, sed do eiusmod tempor incididunt ut labore et dolore magna aliqua. Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>A huggie hoop that sits close to the lobe, with a hinged clasp and polished finish. Comprised of 14K gold, this earring has a width of 1.5 millimetres, diameter of 10 millimetres and weighs 1.4 grams.</t>
+          <t>Duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur. Excepteur sint occaecat cupidatat non proident, sunt in culpa qui officia deserunt mollit anim id est laborum.</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>A huggie hoop that sits close to the lobe, with a hinged clasp and polished finish. Comprised of 14K gold, this earring has a width of 1.5 millimetres, diameter of 12 millimetres and weighs 1.4 grams.</t>
+          <t>Sed ut perspiciatis unde omnis iste natus error sit voluptatem accusantium doloremque laudantium, totam rem aperiam. Nemo enim ipsam voluptatem quia voluptas sit aspernatur aut odit aut fugit, sed quia consequuntur magni dolores.</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>A huggie hoop that sits close to the lobe, with a hinged clasp and polished finish. Comprised of 14K gold, this earring has a width of 1.5 millimetres, diameter of 14 millimetres and weighs 1.4 grams.</t>
+          <t>Lorem ipsum dolor sit amet, consectetur adipiscing elit, sed do eiusmod tempor incididunt ut labore et dolore magna aliqua. Ut enim ad minim veniam, quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>A huggie hoop that sits close to the lobe, with a hinged clasp and polished finish. Comprised of 14K gold, this earring has a width of 1.5 millimetres, diameter of 16 millimetres and weighs 1.4 grams.</t>
+          <t>Duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur. Excepteur sint occaecat cupidatat non proident, sunt in culpa qui officia deserunt mollit anim id est laborum.</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">

</xml_diff>